<commit_message>
Add self-serve signup over the API, and fix a silent blank in scalar sections
A section over a truthy scalar pushed `undefined` as the scope, so {#note}{.}{/note}
rendered empty with no error - exactly the silent blank this product exists to
prevent. Mustache's own semantics are to push the scalar itself; now we do.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_018KEKXsLNnUHdwnAGmnMsHj
</commit_message>
<xml_diff>
--- a/fixtures/textbox.xlsx
+++ b/fixtures/textbox.xlsx
@@ -20,9 +20,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
   <si>
     <t xml:space="preserve">Cell tag {title}</t>
+  </si>
+  <si>
+    <t xml:space="preserve">{%badge}</t>
   </si>
 </sst>
 </file>
@@ -200,12 +203,15 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1"/>
+  <dimension ref="A1:B1"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="0" t="s">
         <v>0</v>
+      </c>
+      <c r="B1" s="0" t="s">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>